<commit_message>
Fixed Flash Chip Footprint
</commit_message>
<xml_diff>
--- a/DSP32-CORE-BOM.xlsx
+++ b/DSP32-CORE-BOM.xlsx
@@ -3,12 +3,17 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="Sheet2" sheetId="2" r:id="rId6"/>
-    <sheet state="visible" name="Sheet3" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="Sheet1" sheetId="1" r:id="rId4"/>
+    <sheet state="visible" name="Sheet2" sheetId="2" r:id="rId5"/>
+    <sheet state="visible" name="Sheet3" sheetId="3" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
+  <extLst>
+    <ext uri="GoogleSheetsCustomDataVersion2">
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId7" roundtripDataChecksum="KW4UqXuMA9fs+6M4ljMbAtZpx95MkkI767v4Wlp1q4s="/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -345,7 +350,7 @@
     <t>W25Q128JVS</t>
   </si>
   <si>
-    <t>Package_SO:SOIC-8_3.9x4.9mm_P1.27mm</t>
+    <t>Package_SO:SOIC-8_5.3x5.3mm_P1.27mm</t>
   </si>
   <si>
     <t>U102</t>
@@ -385,7 +390,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -418,7 +423,6 @@
     <font>
       <color theme="1"/>
       <name val="Calibri"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <color theme="1"/>
@@ -429,6 +433,11 @@
       <sz val="11.0"/>
       <color rgb="FF800080"/>
       <name val="SimSun"/>
+    </font>
+    <font>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10.0"/>
@@ -492,7 +501,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
     </xf>
@@ -503,7 +512,7 @@
       <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+      <alignment horizontal="center" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="1" fillId="2" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
       <alignment horizontal="center" vertical="center"/>
@@ -515,19 +524,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
     <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="bottom"/>
-    </xf>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="center"/>
@@ -535,7 +535,7 @@
     <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
-    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -547,10 +547,10 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
@@ -559,13 +559,13 @@
     <xf borderId="0" fillId="0" fontId="6" numFmtId="49" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf borderId="0" fillId="0" fontId="10" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -615,10 +615,6 @@
 
 <file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1021,8 +1017,8 @@
       <c r="C7" s="7">
         <v>2.0</v>
       </c>
-      <c r="D7" s="8"/>
-      <c r="E7" s="9" t="s">
+      <c r="D7" s="7"/>
+      <c r="E7" s="7" t="s">
         <v>11</v>
       </c>
       <c r="F7" s="7" t="s">
@@ -1031,8 +1027,8 @@
       <c r="G7" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H7" s="8"/>
-      <c r="I7" s="8"/>
+      <c r="H7" s="7"/>
+      <c r="I7" s="7"/>
       <c r="J7" s="1"/>
       <c r="K7" s="1"/>
       <c r="L7" s="1"/>
@@ -1061,7 +1057,7 @@
       <c r="C8" s="7">
         <v>5.0</v>
       </c>
-      <c r="D8" s="8"/>
+      <c r="D8" s="7"/>
       <c r="E8" s="7" t="s">
         <v>15</v>
       </c>
@@ -1071,8 +1067,8 @@
       <c r="G8" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H8" s="8"/>
-      <c r="I8" s="8"/>
+      <c r="H8" s="7"/>
+      <c r="I8" s="7"/>
       <c r="J8" s="1"/>
       <c r="K8" s="1"/>
       <c r="L8" s="1"/>
@@ -1101,7 +1097,7 @@
       <c r="C9" s="7">
         <v>4.0</v>
       </c>
-      <c r="D9" s="8"/>
+      <c r="D9" s="7"/>
       <c r="E9" s="7" t="s">
         <v>18</v>
       </c>
@@ -1111,8 +1107,8 @@
       <c r="G9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H9" s="8"/>
-      <c r="I9" s="8"/>
+      <c r="H9" s="7"/>
+      <c r="I9" s="7"/>
       <c r="J9" s="1"/>
       <c r="K9" s="1"/>
       <c r="L9" s="1"/>
@@ -1141,8 +1137,8 @@
       <c r="C10" s="7">
         <v>11.0</v>
       </c>
-      <c r="D10" s="8"/>
-      <c r="E10" s="9" t="s">
+      <c r="D10" s="7"/>
+      <c r="E10" s="7" t="s">
         <v>21</v>
       </c>
       <c r="F10" s="7" t="s">
@@ -1151,8 +1147,8 @@
       <c r="G10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H10" s="8"/>
-      <c r="I10" s="8"/>
+      <c r="H10" s="7"/>
+      <c r="I10" s="7"/>
       <c r="J10" s="1"/>
       <c r="K10" s="1"/>
       <c r="L10" s="1"/>
@@ -1181,8 +1177,8 @@
       <c r="C11" s="7">
         <v>2.0</v>
       </c>
-      <c r="D11" s="8"/>
-      <c r="E11" s="9" t="s">
+      <c r="D11" s="7"/>
+      <c r="E11" s="7" t="s">
         <v>24</v>
       </c>
       <c r="F11" s="7" t="s">
@@ -1191,8 +1187,8 @@
       <c r="G11" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H11" s="8"/>
-      <c r="I11" s="8"/>
+      <c r="H11" s="7"/>
+      <c r="I11" s="7"/>
       <c r="J11" s="1"/>
       <c r="K11" s="1"/>
       <c r="L11" s="1"/>
@@ -1221,8 +1217,8 @@
       <c r="C12" s="7">
         <v>1.0</v>
       </c>
-      <c r="D12" s="8"/>
-      <c r="E12" s="9" t="s">
+      <c r="D12" s="7"/>
+      <c r="E12" s="7" t="s">
         <v>27</v>
       </c>
       <c r="F12" s="7" t="s">
@@ -1231,8 +1227,8 @@
       <c r="G12" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H12" s="8"/>
-      <c r="I12" s="8"/>
+      <c r="H12" s="7"/>
+      <c r="I12" s="7"/>
       <c r="J12" s="1"/>
       <c r="K12" s="1"/>
       <c r="L12" s="1"/>
@@ -1261,7 +1257,7 @@
       <c r="C13" s="7">
         <v>2.0</v>
       </c>
-      <c r="D13" s="8"/>
+      <c r="D13" s="7"/>
       <c r="E13" s="7" t="s">
         <v>30</v>
       </c>
@@ -1271,8 +1267,8 @@
       <c r="G13" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="H13" s="8"/>
-      <c r="I13" s="8"/>
+      <c r="H13" s="7"/>
+      <c r="I13" s="7"/>
       <c r="J13" s="1"/>
       <c r="K13" s="1"/>
       <c r="L13" s="1"/>
@@ -1301,8 +1297,8 @@
       <c r="C14" s="7">
         <v>2.0</v>
       </c>
-      <c r="D14" s="8"/>
-      <c r="E14" s="10" t="s">
+      <c r="D14" s="7"/>
+      <c r="E14" s="8" t="s">
         <v>33</v>
       </c>
       <c r="F14" s="7" t="s">
@@ -1311,8 +1307,8 @@
       <c r="G14" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="H14" s="8"/>
-      <c r="I14" s="8"/>
+      <c r="H14" s="7"/>
+      <c r="I14" s="7"/>
       <c r="J14" s="1"/>
       <c r="K14" s="1"/>
       <c r="L14" s="1"/>
@@ -1341,8 +1337,8 @@
       <c r="C15" s="7">
         <v>2.0</v>
       </c>
-      <c r="D15" s="8"/>
-      <c r="E15" s="10" t="s">
+      <c r="D15" s="7"/>
+      <c r="E15" s="8" t="s">
         <v>37</v>
       </c>
       <c r="F15" s="7" t="s">
@@ -1351,8 +1347,8 @@
       <c r="G15" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="H15" s="8"/>
-      <c r="I15" s="8"/>
+      <c r="H15" s="7"/>
+      <c r="I15" s="7"/>
       <c r="J15" s="1"/>
       <c r="K15" s="1"/>
       <c r="L15" s="1"/>
@@ -1381,7 +1377,7 @@
       <c r="C16" s="7">
         <v>1.0</v>
       </c>
-      <c r="D16" s="8"/>
+      <c r="D16" s="7"/>
       <c r="E16" s="7" t="s">
         <v>41</v>
       </c>
@@ -1391,8 +1387,8 @@
       <c r="G16" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="H16" s="8"/>
-      <c r="I16" s="8"/>
+      <c r="H16" s="7"/>
+      <c r="I16" s="7"/>
       <c r="J16" s="1"/>
       <c r="K16" s="1"/>
       <c r="L16" s="1"/>
@@ -1421,8 +1417,8 @@
       <c r="C17" s="7">
         <v>1.0</v>
       </c>
-      <c r="D17" s="8"/>
-      <c r="E17" s="10" t="s">
+      <c r="D17" s="7"/>
+      <c r="E17" s="8" t="s">
         <v>45</v>
       </c>
       <c r="F17" s="7" t="s">
@@ -1431,8 +1427,8 @@
       <c r="G17" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="H17" s="8"/>
-      <c r="I17" s="8"/>
+      <c r="H17" s="7"/>
+      <c r="I17" s="7"/>
       <c r="J17" s="1"/>
       <c r="K17" s="1"/>
       <c r="L17" s="1"/>
@@ -1461,15 +1457,15 @@
       <c r="C18" s="7">
         <v>2.0</v>
       </c>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
       <c r="F18" s="7" t="s">
         <v>49</v>
       </c>
       <c r="G18" s="7" t="s">
         <v>50</v>
       </c>
-      <c r="H18" s="8"/>
+      <c r="H18" s="7"/>
       <c r="I18" s="7" t="s">
         <v>51</v>
       </c>
@@ -1501,8 +1497,8 @@
       <c r="C19" s="7">
         <v>2.0</v>
       </c>
-      <c r="D19" s="8"/>
-      <c r="E19" s="9" t="s">
+      <c r="D19" s="7"/>
+      <c r="E19" s="7" t="s">
         <v>53</v>
       </c>
       <c r="F19" s="7" t="s">
@@ -1511,8 +1507,8 @@
       <c r="G19" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="H19" s="8"/>
-      <c r="I19" s="8"/>
+      <c r="H19" s="7"/>
+      <c r="I19" s="7"/>
       <c r="J19" s="1"/>
       <c r="K19" s="1"/>
       <c r="L19" s="1"/>
@@ -1541,7 +1537,7 @@
       <c r="C20" s="7">
         <v>4.0</v>
       </c>
-      <c r="D20" s="8"/>
+      <c r="D20" s="7"/>
       <c r="E20" s="7" t="s">
         <v>57</v>
       </c>
@@ -1551,8 +1547,8 @@
       <c r="G20" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="H20" s="8"/>
-      <c r="I20" s="8"/>
+      <c r="H20" s="7"/>
+      <c r="I20" s="7"/>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
       <c r="L20" s="1"/>
@@ -1581,7 +1577,7 @@
       <c r="C21" s="7">
         <v>2.0</v>
       </c>
-      <c r="D21" s="8"/>
+      <c r="D21" s="7"/>
       <c r="E21" s="7" t="s">
         <v>60</v>
       </c>
@@ -1591,8 +1587,8 @@
       <c r="G21" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="H21" s="8"/>
-      <c r="I21" s="8"/>
+      <c r="H21" s="7"/>
+      <c r="I21" s="7"/>
       <c r="J21" s="1"/>
       <c r="K21" s="1"/>
       <c r="L21" s="1"/>
@@ -1621,8 +1617,8 @@
       <c r="C22" s="7">
         <v>6.0</v>
       </c>
-      <c r="D22" s="8"/>
-      <c r="E22" s="10" t="s">
+      <c r="D22" s="7"/>
+      <c r="E22" s="8" t="s">
         <v>63</v>
       </c>
       <c r="F22" s="7" t="s">
@@ -1631,8 +1627,8 @@
       <c r="G22" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="H22" s="8"/>
-      <c r="I22" s="8"/>
+      <c r="H22" s="7"/>
+      <c r="I22" s="7"/>
       <c r="J22" s="1"/>
       <c r="K22" s="1"/>
       <c r="L22" s="1"/>
@@ -1661,8 +1657,8 @@
       <c r="C23" s="7">
         <v>1.0</v>
       </c>
-      <c r="D23" s="8"/>
-      <c r="E23" s="11" t="s">
+      <c r="D23" s="7"/>
+      <c r="E23" s="8" t="s">
         <v>66</v>
       </c>
       <c r="F23" s="7" t="s">
@@ -1671,8 +1667,8 @@
       <c r="G23" s="7" t="s">
         <v>55</v>
       </c>
-      <c r="H23" s="8"/>
-      <c r="I23" s="8"/>
+      <c r="H23" s="7"/>
+      <c r="I23" s="7"/>
       <c r="J23" s="1"/>
       <c r="K23" s="1"/>
       <c r="L23" s="1"/>
@@ -1701,8 +1697,8 @@
       <c r="C24" s="7">
         <v>2.0</v>
       </c>
-      <c r="D24" s="8"/>
-      <c r="E24" s="10" t="s">
+      <c r="D24" s="7"/>
+      <c r="E24" s="8" t="s">
         <v>69</v>
       </c>
       <c r="F24" s="7" t="s">
@@ -1711,8 +1707,8 @@
       <c r="G24" s="7" t="s">
         <v>71</v>
       </c>
-      <c r="H24" s="8"/>
-      <c r="I24" s="8"/>
+      <c r="H24" s="7"/>
+      <c r="I24" s="7"/>
       <c r="J24" s="1"/>
       <c r="K24" s="1"/>
       <c r="L24" s="1"/>
@@ -1741,8 +1737,8 @@
       <c r="C25" s="7">
         <v>1.0</v>
       </c>
-      <c r="D25" s="8"/>
-      <c r="E25" s="10" t="s">
+      <c r="D25" s="7"/>
+      <c r="E25" s="8" t="s">
         <v>73</v>
       </c>
       <c r="F25" s="7" t="s">
@@ -1751,8 +1747,8 @@
       <c r="G25" s="7" t="s">
         <v>75</v>
       </c>
-      <c r="H25" s="8"/>
-      <c r="I25" s="8"/>
+      <c r="H25" s="7"/>
+      <c r="I25" s="7"/>
       <c r="J25" s="1"/>
       <c r="K25" s="1"/>
       <c r="L25" s="1"/>
@@ -1781,8 +1777,8 @@
       <c r="C26" s="7">
         <v>1.0</v>
       </c>
-      <c r="D26" s="8"/>
-      <c r="E26" s="10" t="s">
+      <c r="D26" s="7"/>
+      <c r="E26" s="8" t="s">
         <v>77</v>
       </c>
       <c r="F26" s="7" t="s">
@@ -1791,25 +1787,25 @@
       <c r="G26" s="7" t="s">
         <v>79</v>
       </c>
-      <c r="H26" s="8"/>
-      <c r="I26" s="8"/>
-      <c r="J26" s="12"/>
-      <c r="K26" s="12"/>
-      <c r="L26" s="12"/>
-      <c r="M26" s="12"/>
-      <c r="N26" s="12"/>
-      <c r="O26" s="12"/>
-      <c r="P26" s="12"/>
-      <c r="Q26" s="12"/>
-      <c r="R26" s="12"/>
-      <c r="S26" s="12"/>
-      <c r="T26" s="12"/>
-      <c r="U26" s="12"/>
-      <c r="V26" s="12"/>
-      <c r="W26" s="12"/>
-      <c r="X26" s="12"/>
-      <c r="Y26" s="12"/>
-      <c r="Z26" s="12"/>
+      <c r="H26" s="7"/>
+      <c r="I26" s="7"/>
+      <c r="J26" s="9"/>
+      <c r="K26" s="9"/>
+      <c r="L26" s="9"/>
+      <c r="M26" s="9"/>
+      <c r="N26" s="9"/>
+      <c r="O26" s="9"/>
+      <c r="P26" s="9"/>
+      <c r="Q26" s="9"/>
+      <c r="R26" s="9"/>
+      <c r="S26" s="9"/>
+      <c r="T26" s="9"/>
+      <c r="U26" s="9"/>
+      <c r="V26" s="9"/>
+      <c r="W26" s="9"/>
+      <c r="X26" s="9"/>
+      <c r="Y26" s="9"/>
+      <c r="Z26" s="9"/>
     </row>
     <row r="27" ht="14.25" customHeight="1">
       <c r="A27" s="7">
@@ -1821,7 +1817,7 @@
       <c r="C27" s="7">
         <v>1.0</v>
       </c>
-      <c r="D27" s="8"/>
+      <c r="D27" s="7"/>
       <c r="E27" s="7" t="s">
         <v>81</v>
       </c>
@@ -1831,8 +1827,8 @@
       <c r="G27" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="H27" s="8"/>
-      <c r="I27" s="8"/>
+      <c r="H27" s="7"/>
+      <c r="I27" s="7"/>
       <c r="J27" s="1"/>
       <c r="K27" s="1"/>
       <c r="L27" s="1"/>
@@ -1861,18 +1857,18 @@
       <c r="C28" s="7">
         <v>1.0</v>
       </c>
-      <c r="D28" s="13"/>
-      <c r="E28" s="14" t="s">
+      <c r="D28" s="10"/>
+      <c r="E28" s="10" t="s">
         <v>85</v>
       </c>
       <c r="F28" s="7" t="s">
         <v>86</v>
       </c>
-      <c r="G28" s="7" t="s">
+      <c r="G28" s="11" t="s">
         <v>87</v>
       </c>
-      <c r="H28" s="13"/>
-      <c r="I28" s="8"/>
+      <c r="H28" s="10"/>
+      <c r="I28" s="7"/>
       <c r="J28" s="1"/>
       <c r="K28" s="1"/>
       <c r="L28" s="1"/>
@@ -1901,8 +1897,8 @@
       <c r="C29" s="7">
         <v>1.0</v>
       </c>
-      <c r="D29" s="13"/>
-      <c r="E29" s="14" t="s">
+      <c r="D29" s="10"/>
+      <c r="E29" s="10" t="s">
         <v>89</v>
       </c>
       <c r="F29" s="7" t="s">
@@ -1911,8 +1907,8 @@
       <c r="G29" s="7" t="s">
         <v>91</v>
       </c>
-      <c r="H29" s="13"/>
-      <c r="I29" s="13"/>
+      <c r="H29" s="10"/>
+      <c r="I29" s="10"/>
       <c r="J29" s="1"/>
       <c r="K29" s="1"/>
       <c r="L29" s="1"/>
@@ -1941,8 +1937,8 @@
       <c r="C30" s="7">
         <v>1.0</v>
       </c>
-      <c r="D30" s="13"/>
-      <c r="E30" s="14" t="s">
+      <c r="D30" s="10"/>
+      <c r="E30" s="10" t="s">
         <v>93</v>
       </c>
       <c r="F30" s="7" t="s">
@@ -1951,8 +1947,8 @@
       <c r="G30" s="7" t="s">
         <v>83</v>
       </c>
-      <c r="H30" s="13"/>
-      <c r="I30" s="13"/>
+      <c r="H30" s="10"/>
+      <c r="I30" s="10"/>
       <c r="J30" s="1"/>
       <c r="K30" s="1"/>
       <c r="L30" s="1"/>
@@ -1981,8 +1977,8 @@
       <c r="C31" s="7">
         <v>1.0</v>
       </c>
-      <c r="D31" s="13"/>
-      <c r="E31" s="10" t="s">
+      <c r="D31" s="10"/>
+      <c r="E31" s="8" t="s">
         <v>96</v>
       </c>
       <c r="F31" s="7" t="s">
@@ -1991,8 +1987,8 @@
       <c r="G31" s="7" t="s">
         <v>98</v>
       </c>
-      <c r="H31" s="13"/>
-      <c r="I31" s="13"/>
+      <c r="H31" s="10"/>
+      <c r="I31" s="10"/>
       <c r="J31" s="1"/>
       <c r="K31" s="1"/>
       <c r="L31" s="1"/>
@@ -2536,15 +2532,15 @@
       <c r="Z50" s="1"/>
     </row>
     <row r="51" ht="14.25" customHeight="1">
-      <c r="A51" s="15"/>
-      <c r="B51" s="16"/>
-      <c r="C51" s="15"/>
-      <c r="D51" s="17"/>
-      <c r="E51" s="16"/>
-      <c r="F51" s="18"/>
-      <c r="G51" s="16"/>
-      <c r="H51" s="19"/>
-      <c r="I51" s="19"/>
+      <c r="A51" s="12"/>
+      <c r="B51" s="13"/>
+      <c r="C51" s="12"/>
+      <c r="D51" s="14"/>
+      <c r="E51" s="13"/>
+      <c r="F51" s="15"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="16"/>
+      <c r="I51" s="16"/>
       <c r="J51" s="1"/>
       <c r="K51" s="1"/>
       <c r="L51" s="1"/>
@@ -2564,15 +2560,15 @@
       <c r="Z51" s="1"/>
     </row>
     <row r="52" ht="14.25" customHeight="1">
-      <c r="A52" s="15"/>
-      <c r="B52" s="16"/>
-      <c r="C52" s="15"/>
-      <c r="D52" s="17"/>
-      <c r="E52" s="16"/>
-      <c r="F52" s="18"/>
-      <c r="G52" s="16"/>
-      <c r="H52" s="19"/>
-      <c r="I52" s="20"/>
+      <c r="A52" s="12"/>
+      <c r="B52" s="13"/>
+      <c r="C52" s="12"/>
+      <c r="D52" s="14"/>
+      <c r="E52" s="13"/>
+      <c r="F52" s="15"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="16"/>
+      <c r="I52" s="17"/>
       <c r="J52" s="1"/>
       <c r="K52" s="1"/>
       <c r="L52" s="1"/>
@@ -2592,15 +2588,15 @@
       <c r="Z52" s="1"/>
     </row>
     <row r="53" ht="14.25" customHeight="1">
-      <c r="A53" s="15"/>
-      <c r="B53" s="16"/>
-      <c r="C53" s="15"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="16"/>
-      <c r="F53" s="18"/>
-      <c r="G53" s="16"/>
-      <c r="H53" s="19"/>
-      <c r="I53" s="19"/>
+      <c r="A53" s="12"/>
+      <c r="B53" s="13"/>
+      <c r="C53" s="12"/>
+      <c r="D53" s="14"/>
+      <c r="E53" s="13"/>
+      <c r="F53" s="15"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="16"/>
+      <c r="I53" s="16"/>
       <c r="J53" s="1"/>
       <c r="K53" s="1"/>
       <c r="L53" s="1"/>
@@ -2620,15 +2616,15 @@
       <c r="Z53" s="1"/>
     </row>
     <row r="54" ht="14.25" customHeight="1">
-      <c r="A54" s="15"/>
-      <c r="B54" s="16"/>
-      <c r="C54" s="15"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="16"/>
-      <c r="F54" s="18"/>
-      <c r="G54" s="16"/>
-      <c r="H54" s="19"/>
-      <c r="I54" s="19"/>
+      <c r="A54" s="12"/>
+      <c r="B54" s="13"/>
+      <c r="C54" s="12"/>
+      <c r="D54" s="14"/>
+      <c r="E54" s="13"/>
+      <c r="F54" s="15"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="16"/>
+      <c r="I54" s="16"/>
       <c r="J54" s="1"/>
       <c r="K54" s="1"/>
       <c r="L54" s="1"/>
@@ -2648,15 +2644,15 @@
       <c r="Z54" s="1"/>
     </row>
     <row r="55" ht="14.25" customHeight="1">
-      <c r="A55" s="15"/>
-      <c r="B55" s="16"/>
-      <c r="C55" s="15"/>
-      <c r="D55" s="17"/>
-      <c r="E55" s="16"/>
-      <c r="F55" s="18"/>
-      <c r="G55" s="16"/>
-      <c r="H55" s="19"/>
-      <c r="I55" s="19"/>
+      <c r="A55" s="12"/>
+      <c r="B55" s="13"/>
+      <c r="C55" s="12"/>
+      <c r="D55" s="14"/>
+      <c r="E55" s="13"/>
+      <c r="F55" s="15"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="16"/>
+      <c r="I55" s="16"/>
       <c r="J55" s="1"/>
       <c r="K55" s="1"/>
       <c r="L55" s="1"/>
@@ -2676,15 +2672,15 @@
       <c r="Z55" s="1"/>
     </row>
     <row r="56" ht="14.25" customHeight="1">
-      <c r="A56" s="15"/>
-      <c r="B56" s="16"/>
-      <c r="C56" s="15"/>
-      <c r="D56" s="17"/>
-      <c r="E56" s="16"/>
-      <c r="F56" s="18"/>
-      <c r="G56" s="21"/>
-      <c r="H56" s="19"/>
-      <c r="I56" s="19"/>
+      <c r="A56" s="12"/>
+      <c r="B56" s="13"/>
+      <c r="C56" s="12"/>
+      <c r="D56" s="14"/>
+      <c r="E56" s="13"/>
+      <c r="F56" s="15"/>
+      <c r="G56" s="18"/>
+      <c r="H56" s="16"/>
+      <c r="I56" s="16"/>
       <c r="J56" s="1"/>
       <c r="K56" s="1"/>
       <c r="L56" s="1"/>
@@ -2704,15 +2700,15 @@
       <c r="Z56" s="1"/>
     </row>
     <row r="57" ht="14.25" customHeight="1">
-      <c r="A57" s="15"/>
-      <c r="B57" s="16"/>
-      <c r="C57" s="15"/>
-      <c r="D57" s="17"/>
-      <c r="E57" s="16"/>
-      <c r="F57" s="18"/>
-      <c r="G57" s="21"/>
-      <c r="H57" s="19"/>
-      <c r="I57" s="19"/>
+      <c r="A57" s="12"/>
+      <c r="B57" s="13"/>
+      <c r="C57" s="12"/>
+      <c r="D57" s="14"/>
+      <c r="E57" s="13"/>
+      <c r="F57" s="15"/>
+      <c r="G57" s="18"/>
+      <c r="H57" s="16"/>
+      <c r="I57" s="16"/>
       <c r="J57" s="1"/>
       <c r="K57" s="1"/>
       <c r="L57" s="1"/>
@@ -2732,15 +2728,15 @@
       <c r="Z57" s="1"/>
     </row>
     <row r="58" ht="14.25" customHeight="1">
-      <c r="A58" s="15"/>
-      <c r="B58" s="16"/>
-      <c r="C58" s="15"/>
-      <c r="D58" s="17"/>
-      <c r="E58" s="16"/>
-      <c r="F58" s="17"/>
-      <c r="G58" s="21"/>
-      <c r="H58" s="19"/>
-      <c r="I58" s="19"/>
+      <c r="A58" s="12"/>
+      <c r="B58" s="13"/>
+      <c r="C58" s="12"/>
+      <c r="D58" s="14"/>
+      <c r="E58" s="13"/>
+      <c r="F58" s="14"/>
+      <c r="G58" s="18"/>
+      <c r="H58" s="16"/>
+      <c r="I58" s="16"/>
       <c r="J58" s="1"/>
       <c r="K58" s="1"/>
       <c r="L58" s="1"/>
@@ -2760,15 +2756,15 @@
       <c r="Z58" s="1"/>
     </row>
     <row r="59" ht="14.25" customHeight="1">
-      <c r="A59" s="15"/>
-      <c r="B59" s="16"/>
-      <c r="C59" s="15"/>
-      <c r="D59" s="17"/>
-      <c r="E59" s="16"/>
-      <c r="F59" s="17"/>
-      <c r="G59" s="21"/>
-      <c r="H59" s="19"/>
-      <c r="I59" s="19"/>
+      <c r="A59" s="12"/>
+      <c r="B59" s="13"/>
+      <c r="C59" s="12"/>
+      <c r="D59" s="14"/>
+      <c r="E59" s="13"/>
+      <c r="F59" s="14"/>
+      <c r="G59" s="18"/>
+      <c r="H59" s="16"/>
+      <c r="I59" s="16"/>
       <c r="J59" s="1"/>
       <c r="K59" s="1"/>
       <c r="L59" s="1"/>
@@ -2788,15 +2784,15 @@
       <c r="Z59" s="1"/>
     </row>
     <row r="60" ht="14.25" customHeight="1">
-      <c r="A60" s="15"/>
-      <c r="B60" s="16"/>
-      <c r="C60" s="15"/>
-      <c r="D60" s="17"/>
-      <c r="E60" s="16"/>
-      <c r="F60" s="17"/>
-      <c r="G60" s="21"/>
-      <c r="H60" s="20"/>
-      <c r="I60" s="20"/>
+      <c r="A60" s="12"/>
+      <c r="B60" s="13"/>
+      <c r="C60" s="12"/>
+      <c r="D60" s="14"/>
+      <c r="E60" s="13"/>
+      <c r="F60" s="14"/>
+      <c r="G60" s="18"/>
+      <c r="H60" s="17"/>
+      <c r="I60" s="17"/>
       <c r="J60" s="1"/>
       <c r="K60" s="1"/>
       <c r="L60" s="1"/>
@@ -2816,15 +2812,15 @@
       <c r="Z60" s="1"/>
     </row>
     <row r="61" ht="14.25" customHeight="1">
-      <c r="A61" s="15"/>
-      <c r="B61" s="16"/>
-      <c r="C61" s="15"/>
-      <c r="D61" s="17"/>
-      <c r="E61" s="16"/>
-      <c r="F61" s="17"/>
-      <c r="G61" s="21"/>
-      <c r="H61" s="19"/>
-      <c r="I61" s="19"/>
+      <c r="A61" s="12"/>
+      <c r="B61" s="13"/>
+      <c r="C61" s="12"/>
+      <c r="D61" s="14"/>
+      <c r="E61" s="13"/>
+      <c r="F61" s="14"/>
+      <c r="G61" s="18"/>
+      <c r="H61" s="16"/>
+      <c r="I61" s="16"/>
       <c r="J61" s="1"/>
       <c r="K61" s="1"/>
       <c r="L61" s="1"/>
@@ -2844,15 +2840,15 @@
       <c r="Z61" s="1"/>
     </row>
     <row r="62" ht="14.25" customHeight="1">
-      <c r="A62" s="15"/>
-      <c r="B62" s="16"/>
-      <c r="C62" s="15"/>
-      <c r="D62" s="17"/>
-      <c r="E62" s="16"/>
-      <c r="F62" s="18"/>
-      <c r="G62" s="21"/>
-      <c r="H62" s="19"/>
-      <c r="I62" s="19"/>
+      <c r="A62" s="12"/>
+      <c r="B62" s="13"/>
+      <c r="C62" s="12"/>
+      <c r="D62" s="14"/>
+      <c r="E62" s="13"/>
+      <c r="F62" s="15"/>
+      <c r="G62" s="18"/>
+      <c r="H62" s="16"/>
+      <c r="I62" s="16"/>
       <c r="J62" s="1"/>
       <c r="K62" s="1"/>
       <c r="L62" s="1"/>
@@ -2872,15 +2868,15 @@
       <c r="Z62" s="1"/>
     </row>
     <row r="63" ht="14.25" customHeight="1">
-      <c r="A63" s="15"/>
-      <c r="B63" s="16"/>
-      <c r="C63" s="15"/>
-      <c r="D63" s="17"/>
-      <c r="E63" s="16"/>
-      <c r="F63" s="17"/>
-      <c r="G63" s="21"/>
-      <c r="H63" s="19"/>
-      <c r="I63" s="19"/>
+      <c r="A63" s="12"/>
+      <c r="B63" s="13"/>
+      <c r="C63" s="12"/>
+      <c r="D63" s="14"/>
+      <c r="E63" s="13"/>
+      <c r="F63" s="14"/>
+      <c r="G63" s="18"/>
+      <c r="H63" s="16"/>
+      <c r="I63" s="16"/>
       <c r="J63" s="1"/>
       <c r="K63" s="1"/>
       <c r="L63" s="1"/>
@@ -2900,15 +2896,15 @@
       <c r="Z63" s="1"/>
     </row>
     <row r="64" ht="14.25" customHeight="1">
-      <c r="A64" s="15"/>
-      <c r="B64" s="16"/>
-      <c r="C64" s="15"/>
-      <c r="D64" s="17"/>
-      <c r="E64" s="16"/>
-      <c r="F64" s="17"/>
-      <c r="G64" s="21"/>
-      <c r="H64" s="19"/>
-      <c r="I64" s="19"/>
+      <c r="A64" s="12"/>
+      <c r="B64" s="13"/>
+      <c r="C64" s="12"/>
+      <c r="D64" s="14"/>
+      <c r="E64" s="13"/>
+      <c r="F64" s="14"/>
+      <c r="G64" s="18"/>
+      <c r="H64" s="16"/>
+      <c r="I64" s="16"/>
       <c r="J64" s="1"/>
       <c r="K64" s="1"/>
       <c r="L64" s="1"/>
@@ -2928,15 +2924,15 @@
       <c r="Z64" s="1"/>
     </row>
     <row r="65" ht="14.25" customHeight="1">
-      <c r="A65" s="15"/>
-      <c r="B65" s="16"/>
-      <c r="C65" s="15"/>
-      <c r="D65" s="17"/>
-      <c r="E65" s="16"/>
-      <c r="F65" s="18"/>
-      <c r="G65" s="21"/>
-      <c r="H65" s="19"/>
-      <c r="I65" s="19"/>
+      <c r="A65" s="12"/>
+      <c r="B65" s="13"/>
+      <c r="C65" s="12"/>
+      <c r="D65" s="14"/>
+      <c r="E65" s="13"/>
+      <c r="F65" s="15"/>
+      <c r="G65" s="18"/>
+      <c r="H65" s="16"/>
+      <c r="I65" s="16"/>
       <c r="J65" s="1"/>
       <c r="K65" s="1"/>
       <c r="L65" s="1"/>
@@ -2956,14 +2952,14 @@
       <c r="Z65" s="1"/>
     </row>
     <row r="66" ht="14.25" customHeight="1">
-      <c r="A66" s="15"/>
-      <c r="B66" s="16"/>
-      <c r="C66" s="15"/>
+      <c r="A66" s="12"/>
+      <c r="B66" s="13"/>
+      <c r="C66" s="12"/>
       <c r="D66" s="1"/>
-      <c r="E66" s="16"/>
+      <c r="E66" s="13"/>
       <c r="F66" s="1"/>
-      <c r="G66" s="16"/>
-      <c r="H66" s="19"/>
+      <c r="G66" s="13"/>
+      <c r="H66" s="16"/>
       <c r="I66" s="1"/>
       <c r="J66" s="1"/>
       <c r="K66" s="1"/>
@@ -2984,14 +2980,14 @@
       <c r="Z66" s="1"/>
     </row>
     <row r="67" ht="14.25" customHeight="1">
-      <c r="A67" s="15"/>
-      <c r="B67" s="16"/>
-      <c r="C67" s="15"/>
+      <c r="A67" s="12"/>
+      <c r="B67" s="13"/>
+      <c r="C67" s="12"/>
       <c r="D67" s="1"/>
-      <c r="E67" s="16"/>
+      <c r="E67" s="13"/>
       <c r="F67" s="1"/>
-      <c r="G67" s="16"/>
-      <c r="H67" s="19"/>
+      <c r="G67" s="13"/>
+      <c r="H67" s="16"/>
       <c r="I67" s="1"/>
       <c r="J67" s="1"/>
       <c r="K67" s="1"/>
@@ -3012,15 +3008,15 @@
       <c r="Z67" s="1"/>
     </row>
     <row r="68" ht="14.25" customHeight="1">
-      <c r="A68" s="15"/>
-      <c r="B68" s="16"/>
-      <c r="C68" s="15"/>
-      <c r="D68" s="22"/>
-      <c r="E68" s="16"/>
-      <c r="F68" s="22"/>
-      <c r="G68" s="16"/>
-      <c r="H68" s="19"/>
-      <c r="I68" s="22"/>
+      <c r="A68" s="12"/>
+      <c r="B68" s="13"/>
+      <c r="C68" s="12"/>
+      <c r="D68" s="19"/>
+      <c r="E68" s="13"/>
+      <c r="F68" s="19"/>
+      <c r="G68" s="13"/>
+      <c r="H68" s="16"/>
+      <c r="I68" s="19"/>
       <c r="J68" s="1"/>
       <c r="K68" s="1"/>
       <c r="L68" s="1"/>
@@ -3040,15 +3036,15 @@
       <c r="Z68" s="1"/>
     </row>
     <row r="69" ht="14.25" customHeight="1">
-      <c r="A69" s="15"/>
-      <c r="B69" s="16"/>
-      <c r="C69" s="15"/>
-      <c r="D69" s="23"/>
-      <c r="E69" s="16"/>
-      <c r="F69" s="23"/>
-      <c r="G69" s="16"/>
-      <c r="H69" s="19"/>
-      <c r="I69" s="23"/>
+      <c r="A69" s="12"/>
+      <c r="B69" s="13"/>
+      <c r="C69" s="12"/>
+      <c r="D69" s="20"/>
+      <c r="E69" s="13"/>
+      <c r="F69" s="20"/>
+      <c r="G69" s="13"/>
+      <c r="H69" s="16"/>
+      <c r="I69" s="20"/>
       <c r="J69" s="1"/>
       <c r="K69" s="1"/>
       <c r="L69" s="1"/>
@@ -3068,15 +3064,15 @@
       <c r="Z69" s="1"/>
     </row>
     <row r="70" ht="14.25" customHeight="1">
-      <c r="A70" s="15"/>
-      <c r="B70" s="16"/>
-      <c r="C70" s="15"/>
-      <c r="D70" s="24"/>
-      <c r="E70" s="16"/>
-      <c r="F70" s="24"/>
-      <c r="G70" s="16"/>
-      <c r="H70" s="19"/>
-      <c r="I70" s="19"/>
+      <c r="A70" s="12"/>
+      <c r="B70" s="13"/>
+      <c r="C70" s="12"/>
+      <c r="D70" s="21"/>
+      <c r="E70" s="13"/>
+      <c r="F70" s="21"/>
+      <c r="G70" s="13"/>
+      <c r="H70" s="16"/>
+      <c r="I70" s="16"/>
       <c r="J70" s="1"/>
       <c r="K70" s="1"/>
       <c r="L70" s="1"/>
@@ -3096,14 +3092,14 @@
       <c r="Z70" s="1"/>
     </row>
     <row r="71" ht="14.25" customHeight="1">
-      <c r="A71" s="15"/>
-      <c r="B71" s="16"/>
-      <c r="C71" s="15"/>
+      <c r="A71" s="12"/>
+      <c r="B71" s="13"/>
+      <c r="C71" s="12"/>
       <c r="D71" s="1"/>
-      <c r="E71" s="16"/>
+      <c r="E71" s="13"/>
       <c r="F71" s="1"/>
-      <c r="G71" s="16"/>
-      <c r="H71" s="19"/>
+      <c r="G71" s="13"/>
+      <c r="H71" s="16"/>
       <c r="I71" s="1"/>
       <c r="J71" s="1"/>
       <c r="K71" s="1"/>
@@ -3124,14 +3120,14 @@
       <c r="Z71" s="1"/>
     </row>
     <row r="72" ht="14.25" customHeight="1">
-      <c r="A72" s="15"/>
-      <c r="B72" s="16"/>
-      <c r="C72" s="15"/>
+      <c r="A72" s="12"/>
+      <c r="B72" s="13"/>
+      <c r="C72" s="12"/>
       <c r="D72" s="1"/>
-      <c r="E72" s="16"/>
+      <c r="E72" s="13"/>
       <c r="F72" s="1"/>
-      <c r="G72" s="16"/>
-      <c r="H72" s="19"/>
+      <c r="G72" s="13"/>
+      <c r="H72" s="16"/>
       <c r="I72" s="1"/>
       <c r="J72" s="1"/>
       <c r="K72" s="1"/>

</xml_diff>